<commit_message>
Cleaning up after changes to linear model
</commit_message>
<xml_diff>
--- a/data/storage_model_inputs.xlsx
+++ b/data/storage_model_inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpsta\code\energy-modeling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D56B9E-031A-4532-9AC2-67BC40615438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C59CEA6C-D4B4-4344-9E77-0C8D3090A9B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{673B1CAA-5412-438B-9658-9FFB10C918E8}"/>
   </bookViews>
@@ -2887,7 +2887,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DA9861-0EC3-4E7D-99FA-4EEDE1B66AA4}">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.26953125" bestFit="1" customWidth="1"/>
@@ -3053,7 +3053,7 @@
         <v>22.5</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4:G13" si="1">F4</f>
+        <f t="shared" ref="G4:G12" si="1">F4</f>
         <v>22.5</v>
       </c>
       <c r="H4">
@@ -3506,58 +3506,6 @@
         <v>0.09</v>
       </c>
       <c r="P12" s="1">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>10</v>
-      </c>
-      <c r="B13">
-        <v>60</v>
-      </c>
-      <c r="C13">
-        <v>2</v>
-      </c>
-      <c r="D13">
-        <v>0.1</v>
-      </c>
-      <c r="E13">
-        <v>0.85</v>
-      </c>
-      <c r="F13">
-        <f t="shared" ref="F13" si="3">(E13-D13)*B13/C13</f>
-        <v>22.5</v>
-      </c>
-      <c r="G13">
-        <f t="shared" si="1"/>
-        <v>22.5</v>
-      </c>
-      <c r="H13">
-        <v>1E-4</v>
-      </c>
-      <c r="I13">
-        <v>0.999</v>
-      </c>
-      <c r="J13" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="K13">
-        <v>1</v>
-      </c>
-      <c r="L13" s="2">
-        <v>5000000</v>
-      </c>
-      <c r="M13" s="1">
-        <v>0.06</v>
-      </c>
-      <c r="N13">
-        <v>20</v>
-      </c>
-      <c r="O13" s="1">
-        <v>0.09</v>
-      </c>
-      <c r="P13" s="1">
         <v>0.03</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated financial model to include NPV of the battery loan, but haven't included in core analysis yet
</commit_message>
<xml_diff>
--- a/data/storage_model_inputs.xlsx
+++ b/data/storage_model_inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpsta\code\energy-modeling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C59CEA6C-D4B4-4344-9E77-0C8D3090A9B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6771E0C-8054-441B-A27C-6DBC8937FE29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{673B1CAA-5412-438B-9658-9FFB10C918E8}"/>
+    <workbookView xWindow="-4470" yWindow="1390" windowWidth="19200" windowHeight="11170" activeTab="1" xr2:uid="{673B1CAA-5412-438B-9658-9FFB10C918E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Time-Series Data" sheetId="1" r:id="rId1"/>
@@ -3020,7 +3020,7 @@
         <v>5000000</v>
       </c>
       <c r="M3" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N3">
         <v>20</v>
@@ -3073,7 +3073,7 @@
         <v>5000000</v>
       </c>
       <c r="M4" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N4">
         <v>20</v>
@@ -3126,7 +3126,7 @@
         <v>5000000</v>
       </c>
       <c r="M5" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N5">
         <v>20</v>
@@ -3179,7 +3179,7 @@
         <v>5000000</v>
       </c>
       <c r="M6" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N6">
         <v>20</v>
@@ -3232,7 +3232,7 @@
         <v>5000000</v>
       </c>
       <c r="M7" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N7">
         <v>20</v>
@@ -3285,7 +3285,7 @@
         <v>5000000</v>
       </c>
       <c r="M8" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N8">
         <v>20</v>
@@ -3338,7 +3338,7 @@
         <v>5000000</v>
       </c>
       <c r="M9" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N9">
         <v>20</v>
@@ -3391,7 +3391,7 @@
         <v>5000000</v>
       </c>
       <c r="M10" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N10">
         <v>20</v>
@@ -3444,7 +3444,7 @@
         <v>5000000</v>
       </c>
       <c r="M11" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N11">
         <v>20</v>
@@ -3497,7 +3497,7 @@
         <v>5000000</v>
       </c>
       <c r="M12" s="1">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="N12">
         <v>20</v>

</xml_diff>